<commit_message>
Correcao VIN: VehicleIdentificationNumber (nao Name) - telas dual search, mapping SAP regenerado
</commit_message>
<xml_diff>
--- a/integracion/GrupoQ_Mapeo_Cargas_SAP_Salesforce.xlsx
+++ b/integracion/GrupoQ_Mapeo_Cargas_SAP_Salesforce.xlsx
@@ -739,461 +739,461 @@
       </c>
       <c r="B4" t="inlineStr" s="6">
         <is>
+          <t xml:space="preserve">Vehicle.VehicleIdentificationNumber</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Text</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">VIN 17 chars (ISO 3779); el punto (.) del re-ingreso queda SOLO en SAP</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">CLAVE DE UPSERT (unicidad de la unidad)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">LISTO</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">CORRECCION 07/08: el VIN vive en VehicleIdentificationNumber (standard), NO en Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">descripcion de la unidad</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="9">
+        <is>
           <t xml:space="preserve">Vehicle.Name</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr" s="6">
+      <c r="C5" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">Name</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">VIN 17 chars (ISO 3779); el punto (.) del re-ingreso queda SOLO en SAP</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">CLAVE DE UPSERT (unique en la org)</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">LISTO</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">identidad de la unidad</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">nº inventario VMS</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Vehicle.StockCode</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Text</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">número de inventario SAP</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">por VIN</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">LISTO</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">re-ingreso usado = MISMO Vehicle, StockCode nuevo (HU-045 D2)</t>
+      <c r="D5" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">nombre descriptivo (marca+modelo) o el VIN, a definir en la carga</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">busqueda por nombre en las pantallas HU-046</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">DEFINIR</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">las pantallas buscan VIN O Name</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr" s="6">
         <is>
+          <t xml:space="preserve">nº inventario VMS</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Vehicle.StockCode</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Text</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">número de inventario SAP</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">por VIN</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">LISTO</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">re-ingreso usado = MISMO Vehicle, StockCode nuevo (HU-045 D2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr" s="6">
+        <is>
           <t xml:space="preserve">id origen</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr" s="6">
+      <c r="B7" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Vehicle.SourceSystemIdentifier</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr" s="6">
+      <c r="C7" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Text</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr" s="6">
+      <c r="D7" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">id del registro en SAP</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr" s="6">
+      <c r="E7" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr" s="6">
+      <c r="F7" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">LISTO</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr" s="6">
+      <c r="G7" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">T18 HU-045</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr" s="9">
+    <row r="8">
+      <c r="A8" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">WERKS del stock</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr" s="9">
+      <c r="B8" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">Vehicle.CurrentOwnerId</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr" s="9">
+      <c r="C8" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">Lookup(Account)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr" s="9">
+      <c r="D8" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">resolver dealer por código de centro</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr" s="9">
+      <c r="E8" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">vía AccountNumber/External ID</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr" s="9">
+      <c r="F8" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">PENDIENTE códigos</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr" s="9">
+      <c r="G8" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">posesión operativa; alimenta cupos demo HU-046</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">marca/modelo/año/versión</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Vehicle.Make/Model/ModelYear/TrimLevel</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Text/Picklist</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">del maestro del vehículo</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">LISTO</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">nativos (D7 HU-045)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr" s="6">
         <is>
+          <t xml:space="preserve">marca/modelo/año/versión</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Vehicle.Make/Model/ModelYear/TrimLevel</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Text/Picklist</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">del maestro del vehículo</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">LISTO</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">nativos (D7 HU-045)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="6">
+        <is>
           <t xml:space="preserve">país</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr" s="6">
+      <c r="B10" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Vehicle.LocationCountry/LocationCountryCode</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr" s="6">
+      <c r="C10" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Text</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr" s="6">
+      <c r="D10" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">país de la unidad</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr" s="6">
+      <c r="E10" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr" s="6">
+      <c r="F10" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">LISTO</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr" s="6">
+      <c r="G10" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">único Location* poblado hoy</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr" s="9">
-        <is>
-          <t xml:space="preserve">sucursal (nombre)</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr" s="9">
-        <is>
-          <t xml:space="preserve">Vehicle.LocationCity</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr" s="9">
-        <is>
-          <t xml:space="preserve">Text</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr" s="9">
-        <is>
-          <t xml:space="preserve">PREMISA DE CARGA: nombre de sucursal igual a lista de cupos</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr" s="9">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr" s="9">
-        <is>
-          <t xml:space="preserve">PREMISA</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr" s="9">
-        <is>
-          <t xml:space="preserve">sin esto no hay derivación automática de sucursal (wire B v2)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr" s="9">
         <is>
+          <t xml:space="preserve">sucursal (nombre)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Vehicle.LocationCity</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">Text</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">PREMISA DE CARGA: nombre de sucursal igual a lista de cupos</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">PREMISA</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr" s="9">
+        <is>
+          <t xml:space="preserve">sin esto no hay derivación automática de sucursal (wire B v2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr" s="9">
+        <is>
           <t xml:space="preserve">estado comercial</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr" s="9">
+      <c r="B12" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">Vehicle.Status</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr" s="9">
+      <c r="C12" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">Picklist</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr" s="9">
+      <c r="D12" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">SOLO estado comercial; stock/bloqueos NO se replican</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr" s="9">
+      <c r="E12" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr" s="9">
+      <c r="F12" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">LISTO</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr" s="9">
+      <c r="G12" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">máquina de estados única (demo/exh/consignación/reparación) — doc con Meli</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">— (no viene de SAP)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Vehicle.LastOdometerReading</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Number</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">km capturado en SF (RN2 HU-045)</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">LISTO</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">NO mapear desde SAP</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr" s="6">
         <is>
+          <t xml:space="preserve">— (no viene de SAP)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Vehicle.LastOdometerReading</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Number</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">km capturado en SF (RN2 HU-045)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">LISTO</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">NO mapear desde SAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr" s="6">
+        <is>
           <t xml:space="preserve">BUKRS del stock</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr" s="6">
+      <c r="B14" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Asset.AccountId</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr" s="6">
+      <c r="C14" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Lookup(Account)</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr" s="6">
+      <c r="D14" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">resolver SOCIEDAD por código</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr" s="6">
+      <c r="E14" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">vía AccountNumber/External ID</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr" s="6">
+      <c r="F14" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">LISTO (códigos soc.)</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr" s="6">
+      <c r="G14" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">dueño contable del par</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr" s="9">
+    <row r="15">
+      <c r="A15" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">LGORT (almacén)</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr" s="9">
+      <c r="B15" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">Asset.LocationId</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr" s="9">
+      <c r="C15" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">Lookup(Location)</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr" s="9">
+      <c r="D15" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">resolver Location por código/nombre de almacén</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr" s="9">
+      <c r="E15" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">ExternalReference de Location</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr" s="9">
+      <c r="F15" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">PENDIENTE</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr" s="9">
+      <c r="G15" t="inlineStr" s="9">
         <is>
           <t xml:space="preserve">Locations no existen aún (T09 — dato del cliente)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">fecha compra original</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Asset.PurchaseDate</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Date</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">LISTO</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">historial HU-045</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">proveedor/entregó</t>
+          <t xml:space="preserve">fecha compra original</t>
         </is>
       </c>
       <c r="B16" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">Asset.AssetProvidedById</t>
+          <t xml:space="preserve">Asset.PurchaseDate</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">Lookup</t>
+          <t xml:space="preserve">Date</t>
         </is>
       </c>
       <c r="D16" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">quién entregó la unidad</t>
+          <t xml:space="preserve">—</t>
         </is>
       </c>
       <c r="E16" t="inlineStr" s="6">
@@ -1208,19 +1208,19 @@
       </c>
       <c r="G16" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">HU-045</t>
+          <t xml:space="preserve">historial HU-045</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">MATNR del vehículo</t>
+          <t xml:space="preserve">proveedor/entregó</t>
         </is>
       </c>
       <c r="B17" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">Asset.Product2Id / VehicleDefinition</t>
+          <t xml:space="preserve">Asset.AssetProvidedById</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="6">
@@ -1230,57 +1230,94 @@
       </c>
       <c r="D17" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">resolver modelo por ProductCode=MATNR</t>
+          <t xml:space="preserve">quién entregó la unidad</t>
         </is>
       </c>
       <c r="E17" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">MATNR</t>
+          <t xml:space="preserve">—</t>
         </is>
       </c>
       <c r="F17" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">LISTO catálogo nuevos</t>
+          <t xml:space="preserve">LISTO</t>
         </is>
       </c>
       <c r="G17" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">usados de terceros: VD genérica "Used Vehicle" (decisión HU-045)</t>
+          <t xml:space="preserve">HU-045</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr" s="6">
         <is>
+          <t xml:space="preserve">MATNR del vehículo</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Asset.Product2Id / VehicleDefinition</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Lookup</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">resolver modelo por ProductCode=MATNR</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">MATNR</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">LISTO catálogo nuevos</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">usados de terceros: VD genérica "Used Vehicle" (decisión HU-045)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr" s="6">
+        <is>
           <t xml:space="preserve">comprador (venta)</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr" s="6">
+      <c r="B19" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">transferencia CurrentOwnerId → cliente + AssetAccountParticipant</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr" s="6">
+      <c r="C19" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr" s="6">
+      <c r="D19" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">proceso de venta, no carga</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr" s="6">
+      <c r="E19" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr" s="6">
+      <c r="F19" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">DISEÑO</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr" s="6">
+      <c r="G19" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">histórico de dueños</t>
         </is>

</xml_diff>